<commit_message>
fix: correct REFramework transaction flow and PDF reading logic
</commit_message>
<xml_diff>
--- a/Data/Output/Invoices.xlsx
+++ b/Data/Output/Invoices.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\development\UiPath\InvoiceProcessing\Data\Output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACDDAF17-E28B-4168-A639-DFCA266294EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D9B1B97-3890-492B-9680-7D80F08F9FB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{B44E2BD4-138A-40BD-A20E-87A4A2A86A1B}"/>
+    <workbookView xWindow="1780" yWindow="1780" windowWidth="14400" windowHeight="7270" xr2:uid="{B44E2BD4-138A-40BD-A20E-87A4A2A86A1B}"/>
   </bookViews>
   <sheets>
     <sheet name="Invoices" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>BillTo</t>
   </si>
@@ -52,6 +52,18 @@
   </si>
   <si>
     <t>Simple Co.</t>
+  </si>
+  <si>
+    <t>Global Ltd</t>
+  </si>
+  <si>
+    <t>Consulting Group</t>
+  </si>
+  <si>
+    <t>Acme Corp</t>
+  </si>
+  <si>
+    <t>Freelancer Studio</t>
   </si>
 </sst>
 </file>
@@ -423,7 +435,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66AC928E-E45A-40CB-A4C8-0D75A3CD64B7}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
@@ -439,12 +451,34 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B4" t="s">
         <v>4</v>
       </c>
-      <c r="C2">
+      <c r="C4">
         <v>120</v>
       </c>
     </row>

</xml_diff>

<commit_message>
resolve transaction handling and dynamic invoice processing issues
</commit_message>
<xml_diff>
--- a/Data/Output/Invoices.xlsx
+++ b/Data/Output/Invoices.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\development\UiPath\InvoiceProcessing\Data\Output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D9B1B97-3890-492B-9680-7D80F08F9FB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48B6FD89-C164-48F8-99DD-B787A3D67DAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1780" yWindow="1780" windowWidth="14400" windowHeight="7270" xr2:uid="{B44E2BD4-138A-40BD-A20E-87A4A2A86A1B}"/>
+    <workbookView minimized="1" xWindow="1780" yWindow="1780" windowWidth="14400" windowHeight="7270" xr2:uid="{B44E2BD4-138A-40BD-A20E-87A4A2A86A1B}"/>
   </bookViews>
   <sheets>
     <sheet name="Invoices" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="13">
   <si>
     <t>BillTo</t>
   </si>
@@ -64,6 +64,18 @@
   </si>
   <si>
     <t>Freelancer Studio</t>
+  </si>
+  <si>
+    <t>Beta Ltd</t>
+  </si>
+  <si>
+    <t>Gamma LLC</t>
+  </si>
+  <si>
+    <t>Delta Inc</t>
+  </si>
+  <si>
+    <t>Epsilon Co</t>
   </si>
 </sst>
 </file>
@@ -435,7 +447,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66AC928E-E45A-40CB-A4C8-0D75A3CD64B7}">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
@@ -451,34 +463,78 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C2">
-        <v>1140</v>
+        <v>640</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B3" t="s">
         <v>8</v>
       </c>
       <c r="C3">
-        <v>550</v>
+        <v>610</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5">
+        <v>990</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B8" t="s">
         <v>4</v>
       </c>
-      <c r="C4">
+      <c r="C8">
         <v>120</v>
       </c>
     </row>

</xml_diff>